<commit_message>
chore(weekly-sync): auto-pull through 2026-08-24
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week34.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week34.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SB" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SB" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,42 +419,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -855,13 +843,13 @@
         <v>371</v>
       </c>
       <c r="F15" t="n">
-        <v>38773</v>
+        <v>38771</v>
       </c>
       <c r="G15" t="n">
-        <v>42169.51</v>
+        <v>39882.23</v>
       </c>
       <c r="H15" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -883,7 +871,7 @@
         <v>1127</v>
       </c>
       <c r="F16" t="n">
-        <v>64557</v>
+        <v>64556</v>
       </c>
       <c r="G16" t="n">
         <v>54692.39</v>
@@ -1079,7 +1067,7 @@
         <v>295</v>
       </c>
       <c r="F23" t="n">
-        <v>28041</v>
+        <v>28039</v>
       </c>
       <c r="G23" t="n">
         <v>10589.83</v>
@@ -1390,10 +1378,10 @@
         <v>9977</v>
       </c>
       <c r="G34" t="n">
-        <v>30908.45</v>
+        <v>35483.87</v>
       </c>
       <c r="H34" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35">
@@ -1418,10 +1406,10 @@
         <v>15243</v>
       </c>
       <c r="G35" t="n">
-        <v>13726.26</v>
+        <v>18301.68</v>
       </c>
       <c r="H35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
@@ -1443,7 +1431,7 @@
         <v>107</v>
       </c>
       <c r="F36" t="n">
-        <v>8701</v>
+        <v>8700</v>
       </c>
       <c r="G36" t="n">
         <v>5252.54</v>
@@ -1527,7 +1515,7 @@
         <v>767</v>
       </c>
       <c r="F39" t="n">
-        <v>144689</v>
+        <v>144687</v>
       </c>
       <c r="G39" t="n">
         <v>10161</v>
@@ -1639,7 +1627,7 @@
         <v>766</v>
       </c>
       <c r="F43" t="n">
-        <v>72766</v>
+        <v>72762</v>
       </c>
       <c r="G43" t="n">
         <v>24490.65</v>
@@ -2171,7 +2159,7 @@
         <v>84</v>
       </c>
       <c r="F62" t="n">
-        <v>17182</v>
+        <v>17181</v>
       </c>
       <c r="G62" t="n">
         <v>3194.07</v>
@@ -2255,7 +2243,7 @@
         <v>220</v>
       </c>
       <c r="F65" t="n">
-        <v>48459</v>
+        <v>48457</v>
       </c>
       <c r="G65" t="n">
         <v>7721.18</v>
@@ -2479,7 +2467,7 @@
         <v>97</v>
       </c>
       <c r="F73" t="n">
-        <v>12026</v>
+        <v>12025</v>
       </c>
       <c r="G73" t="n">
         <v>2710.16</v>
@@ -2591,7 +2579,7 @@
         <v>402</v>
       </c>
       <c r="F77" t="n">
-        <v>81457</v>
+        <v>81456</v>
       </c>
       <c r="G77" t="n">
         <v>23724.58</v>
@@ -2731,7 +2719,7 @@
         <v>577</v>
       </c>
       <c r="F82" t="n">
-        <v>105676</v>
+        <v>105675</v>
       </c>
       <c r="G82" t="n">
         <v>11268.64</v>
@@ -2759,7 +2747,7 @@
         <v>1927</v>
       </c>
       <c r="F83" t="n">
-        <v>276932</v>
+        <v>276930</v>
       </c>
       <c r="G83" t="n">
         <v>10925.41</v>
@@ -2787,7 +2775,7 @@
         <v>28</v>
       </c>
       <c r="F84" t="n">
-        <v>17569</v>
+        <v>17567</v>
       </c>
       <c r="G84" t="n">
         <v>1007.63</v>
@@ -2927,7 +2915,7 @@
         <v>72</v>
       </c>
       <c r="F89" t="n">
-        <v>11081</v>
+        <v>11079</v>
       </c>
       <c r="G89" t="n">
         <v>0</v>
@@ -2955,7 +2943,7 @@
         <v>76</v>
       </c>
       <c r="F90" t="n">
-        <v>10480</v>
+        <v>10479</v>
       </c>
       <c r="G90" t="n">
         <v>0</v>
@@ -2977,19 +2965,19 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>421.67</v>
+        <v>417.49</v>
       </c>
       <c r="E91" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F91" t="n">
-        <v>15032</v>
+        <v>15031</v>
       </c>
       <c r="G91" t="n">
-        <v>0</v>
+        <v>3388.98</v>
       </c>
       <c r="H91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -3123,13 +3111,13 @@
         <v>475</v>
       </c>
       <c r="F96" t="n">
-        <v>90637</v>
+        <v>90636</v>
       </c>
       <c r="G96" t="n">
-        <v>6776.28</v>
+        <v>8470.35</v>
       </c>
       <c r="H96" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="97">
@@ -3151,7 +3139,7 @@
         <v>137</v>
       </c>
       <c r="F97" t="n">
-        <v>28404</v>
+        <v>28403</v>
       </c>
       <c r="G97" t="n">
         <v>9809.310000000001</v>
@@ -3269,7 +3257,7 @@
         <v>26601.66</v>
       </c>
       <c r="H101" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="102">
@@ -3291,7 +3279,7 @@
         <v>1921</v>
       </c>
       <c r="F102" t="n">
-        <v>248073</v>
+        <v>248072</v>
       </c>
       <c r="G102" t="n">
         <v>14065.25</v>
@@ -3487,7 +3475,7 @@
         <v>82</v>
       </c>
       <c r="F109" t="n">
-        <v>13680</v>
+        <v>13679</v>
       </c>
       <c r="G109" t="n">
         <v>0</v>
@@ -3599,7 +3587,7 @@
         <v>236</v>
       </c>
       <c r="F113" t="n">
-        <v>38618</v>
+        <v>38617</v>
       </c>
       <c r="G113" t="n">
         <v>3641.52</v>
@@ -3677,13 +3665,13 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>5026.71</v>
+        <v>5024.29</v>
       </c>
       <c r="E116" t="n">
-        <v>1854</v>
+        <v>1853</v>
       </c>
       <c r="F116" t="n">
-        <v>237646</v>
+        <v>237644</v>
       </c>
       <c r="G116" t="n">
         <v>43722.04</v>
@@ -3733,13 +3721,13 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>1772.4</v>
+        <v>1769.5</v>
       </c>
       <c r="E118" t="n">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F118" t="n">
-        <v>41092</v>
+        <v>41091</v>
       </c>
       <c r="G118" t="n">
         <v>5930.5</v>
@@ -3798,10 +3786,10 @@
         <v>5930</v>
       </c>
       <c r="G120" t="n">
-        <v>12710.16</v>
+        <v>19065.24</v>
       </c>
       <c r="H120" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="121">
@@ -3823,7 +3811,7 @@
         <v>295</v>
       </c>
       <c r="F121" t="n">
-        <v>45575</v>
+        <v>45574</v>
       </c>
       <c r="G121" t="n">
         <v>15252.54</v>
@@ -3851,7 +3839,7 @@
         <v>507</v>
       </c>
       <c r="F122" t="n">
-        <v>59006</v>
+        <v>59005</v>
       </c>
       <c r="G122" t="n">
         <v>6355.08</v>
@@ -3873,13 +3861,13 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1389.89</v>
+        <v>1388.4</v>
       </c>
       <c r="E123" t="n">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F123" t="n">
-        <v>43360</v>
+        <v>43358</v>
       </c>
       <c r="G123" t="n">
         <v>59738.97</v>
@@ -3929,13 +3917,13 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>7989.15</v>
+        <v>7975.38</v>
       </c>
       <c r="E125" t="n">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="F125" t="n">
-        <v>28970</v>
+        <v>28969</v>
       </c>
       <c r="G125" t="n">
         <v>26092.33</v>
@@ -4019,7 +4007,7 @@
         <v>417</v>
       </c>
       <c r="F128" t="n">
-        <v>33923</v>
+        <v>33922</v>
       </c>
       <c r="G128" t="n">
         <v>14659.32</v>
@@ -4134,10 +4122,10 @@
         <v>40177</v>
       </c>
       <c r="G132" t="n">
-        <v>16093.2</v>
+        <v>17702.52</v>
       </c>
       <c r="H132" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="133">
@@ -4159,7 +4147,7 @@
         <v>284</v>
       </c>
       <c r="F133" t="n">
-        <v>51380</v>
+        <v>51379</v>
       </c>
       <c r="G133" t="n">
         <v>6437.28</v>
@@ -4190,10 +4178,10 @@
         <v>20308</v>
       </c>
       <c r="G134" t="n">
-        <v>6861.87</v>
+        <v>4574.58</v>
       </c>
       <c r="H134" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="135">
@@ -4439,7 +4427,7 @@
         <v>359</v>
       </c>
       <c r="F143" t="n">
-        <v>29617</v>
+        <v>29616</v>
       </c>
       <c r="G143" t="n">
         <v>20362.72</v>
@@ -4467,7 +4455,7 @@
         <v>257</v>
       </c>
       <c r="F144" t="n">
-        <v>22624</v>
+        <v>22623</v>
       </c>
       <c r="G144" t="n">
         <v>12200.85</v>
@@ -4495,7 +4483,7 @@
         <v>193</v>
       </c>
       <c r="F145" t="n">
-        <v>73975</v>
+        <v>73974</v>
       </c>
       <c r="G145" t="n">
         <v>3769.49</v>
@@ -4635,7 +4623,7 @@
         <v>265</v>
       </c>
       <c r="F150" t="n">
-        <v>118318</v>
+        <v>118314</v>
       </c>
       <c r="G150" t="n">
         <v>11564.39</v>
@@ -5195,7 +5183,7 @@
         <v>1062</v>
       </c>
       <c r="F170" t="n">
-        <v>79943</v>
+        <v>79942</v>
       </c>
       <c r="G170" t="n">
         <v>33894.92</v>
@@ -5307,7 +5295,7 @@
         <v>601</v>
       </c>
       <c r="F174" t="n">
-        <v>67508</v>
+        <v>67507</v>
       </c>
       <c r="G174" t="n">
         <v>17794.08</v>
@@ -5503,7 +5491,7 @@
         <v>209</v>
       </c>
       <c r="F181" t="n">
-        <v>188833</v>
+        <v>188832</v>
       </c>
       <c r="G181" t="n">
         <v>0</v>
@@ -5534,10 +5522,10 @@
         <v>19504</v>
       </c>
       <c r="G182" t="n">
-        <v>1100.85</v>
+        <v>2201.7</v>
       </c>
       <c r="H182" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="183">
@@ -5895,7 +5883,7 @@
         <v>69</v>
       </c>
       <c r="F195" t="n">
-        <v>6050</v>
+        <v>6049</v>
       </c>
       <c r="G195" t="n">
         <v>0</v>
@@ -5951,7 +5939,7 @@
         <v>136</v>
       </c>
       <c r="F197" t="n">
-        <v>24395</v>
+        <v>24394</v>
       </c>
       <c r="G197" t="n">
         <v>0</v>
@@ -6038,10 +6026,10 @@
         <v>8528</v>
       </c>
       <c r="G200" t="n">
-        <v>8532.210000000001</v>
+        <v>11726.28</v>
       </c>
       <c r="H200" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="201">
@@ -6371,7 +6359,7 @@
         <v>533</v>
       </c>
       <c r="F212" t="n">
-        <v>83813</v>
+        <v>83812</v>
       </c>
       <c r="G212" t="n">
         <v>0</v>
@@ -6455,7 +6443,7 @@
         <v>544</v>
       </c>
       <c r="F215" t="n">
-        <v>114209</v>
+        <v>114203</v>
       </c>
       <c r="G215" t="n">
         <v>3048.3</v>
@@ -6483,7 +6471,7 @@
         <v>72</v>
       </c>
       <c r="F216" t="n">
-        <v>9144</v>
+        <v>9143</v>
       </c>
       <c r="G216" t="n">
         <v>5294.059999999999</v>
@@ -6514,10 +6502,10 @@
         <v>7809</v>
       </c>
       <c r="G217" t="n">
-        <v>1609.32</v>
+        <v>2879.66</v>
       </c>
       <c r="H217" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="218">
@@ -6539,7 +6527,7 @@
         <v>150</v>
       </c>
       <c r="F218" t="n">
-        <v>11736</v>
+        <v>11734</v>
       </c>
       <c r="G218" t="n">
         <v>21250.86</v>
@@ -6567,7 +6555,7 @@
         <v>32</v>
       </c>
       <c r="F219" t="n">
-        <v>3404</v>
+        <v>3403</v>
       </c>
       <c r="G219" t="n">
         <v>0</v>
@@ -6651,7 +6639,7 @@
         <v>38</v>
       </c>
       <c r="F222" t="n">
-        <v>6417</v>
+        <v>6416</v>
       </c>
       <c r="G222" t="n">
         <v>10407.62</v>
@@ -6757,13 +6745,13 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>1764.02</v>
+        <v>1761.29</v>
       </c>
       <c r="E226" t="n">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F226" t="n">
-        <v>27543</v>
+        <v>27540</v>
       </c>
       <c r="G226" t="n">
         <v>7709.32</v>
@@ -6791,7 +6779,7 @@
         <v>893</v>
       </c>
       <c r="F227" t="n">
-        <v>64566</v>
+        <v>64561</v>
       </c>
       <c r="G227" t="n">
         <v>6701.690000000001</v>
@@ -6931,13 +6919,13 @@
         <v>156</v>
       </c>
       <c r="F232" t="n">
-        <v>13338</v>
+        <v>13336</v>
       </c>
       <c r="G232" t="n">
-        <v>19300.85</v>
+        <v>22520.34</v>
       </c>
       <c r="H232" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="233">
@@ -6959,7 +6947,7 @@
         <v>61</v>
       </c>
       <c r="F233" t="n">
-        <v>7655</v>
+        <v>7652</v>
       </c>
       <c r="G233" t="n">
         <v>5590.68</v>
@@ -6987,7 +6975,7 @@
         <v>526</v>
       </c>
       <c r="F234" t="n">
-        <v>51590</v>
+        <v>51587</v>
       </c>
       <c r="G234" t="n">
         <v>0</v>
@@ -7015,7 +7003,7 @@
         <v>74</v>
       </c>
       <c r="F235" t="n">
-        <v>17307</v>
+        <v>17306</v>
       </c>
       <c r="G235" t="n">
         <v>18333.04</v>
@@ -7043,7 +7031,7 @@
         <v>169</v>
       </c>
       <c r="F236" t="n">
-        <v>18632</v>
+        <v>18631</v>
       </c>
       <c r="G236" t="n">
         <v>2626.27</v>
@@ -7071,13 +7059,13 @@
         <v>585</v>
       </c>
       <c r="F237" t="n">
-        <v>42701</v>
+        <v>42699</v>
       </c>
       <c r="G237" t="n">
-        <v>29984.67</v>
+        <v>31339.75</v>
       </c>
       <c r="H237" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="238">
@@ -7211,7 +7199,7 @@
         <v>10</v>
       </c>
       <c r="F242" t="n">
-        <v>2084</v>
+        <v>2083</v>
       </c>
       <c r="G242" t="n">
         <v>0</v>
@@ -7267,7 +7255,7 @@
         <v>27</v>
       </c>
       <c r="F244" t="n">
-        <v>3694</v>
+        <v>3693</v>
       </c>
       <c r="G244" t="n">
         <v>5931.36</v>
@@ -7295,7 +7283,7 @@
         <v>10</v>
       </c>
       <c r="F245" t="n">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="G245" t="n">
         <v>3195.96</v>
@@ -7351,13 +7339,13 @@
         <v>487</v>
       </c>
       <c r="F247" t="n">
-        <v>41522</v>
+        <v>41520</v>
       </c>
       <c r="G247" t="n">
-        <v>19036.48</v>
+        <v>19544.11</v>
       </c>
       <c r="H247" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="248">
@@ -7379,7 +7367,7 @@
         <v>412</v>
       </c>
       <c r="F248" t="n">
-        <v>37935</v>
+        <v>37934</v>
       </c>
       <c r="G248" t="n">
         <v>9144.9</v>
@@ -7435,7 +7423,7 @@
         <v>94</v>
       </c>
       <c r="F250" t="n">
-        <v>15888</v>
+        <v>15885</v>
       </c>
       <c r="G250" t="n">
         <v>4066.95</v>
@@ -7457,13 +7445,13 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>322.36</v>
+        <v>316.07</v>
       </c>
       <c r="E251" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F251" t="n">
-        <v>5401</v>
+        <v>5398</v>
       </c>
       <c r="G251" t="n">
         <v>0</v>
@@ -7485,13 +7473,13 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>830.5899999999999</v>
+        <v>817.51</v>
       </c>
       <c r="E252" t="n">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F252" t="n">
-        <v>10961</v>
+        <v>10959</v>
       </c>
       <c r="G252" t="n">
         <v>21139.82</v>
@@ -7659,7 +7647,7 @@
         <v>38</v>
       </c>
       <c r="F258" t="n">
-        <v>4891</v>
+        <v>4889</v>
       </c>
       <c r="G258" t="n">
         <v>2540.68</v>
@@ -7681,13 +7669,13 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>1741.69</v>
+        <v>1729.46</v>
       </c>
       <c r="E259" t="n">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="F259" t="n">
-        <v>20772</v>
+        <v>20768</v>
       </c>
       <c r="G259" t="n">
         <v>25421.19</v>
@@ -7743,7 +7731,7 @@
         <v>174</v>
       </c>
       <c r="F261" t="n">
-        <v>22400</v>
+        <v>22397</v>
       </c>
       <c r="G261" t="n">
         <v>4616.940000000001</v>
@@ -7771,7 +7759,7 @@
         <v>18</v>
       </c>
       <c r="F262" t="n">
-        <v>3550</v>
+        <v>3547</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
@@ -7911,7 +7899,7 @@
         <v>603</v>
       </c>
       <c r="F267" t="n">
-        <v>27560</v>
+        <v>27558</v>
       </c>
       <c r="G267" t="n">
         <v>28337.26</v>
@@ -7967,7 +7955,7 @@
         <v>214</v>
       </c>
       <c r="F269" t="n">
-        <v>12462</v>
+        <v>12459</v>
       </c>
       <c r="G269" t="n">
         <v>11693.22</v>
@@ -7995,7 +7983,7 @@
         <v>383</v>
       </c>
       <c r="F270" t="n">
-        <v>34673</v>
+        <v>34671</v>
       </c>
       <c r="G270" t="n">
         <v>29995.77</v>
@@ -8045,13 +8033,13 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>2227.4</v>
+        <v>2225.92</v>
       </c>
       <c r="E272" t="n">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F272" t="n">
-        <v>35404</v>
+        <v>35403</v>
       </c>
       <c r="G272" t="n">
         <v>14404.23</v>
@@ -8107,7 +8095,7 @@
         <v>124</v>
       </c>
       <c r="F274" t="n">
-        <v>8915</v>
+        <v>8913</v>
       </c>
       <c r="G274" t="n">
         <v>27878.81</v>
@@ -8194,10 +8182,10 @@
         <v>7199</v>
       </c>
       <c r="G277" t="n">
-        <v>4413.54</v>
+        <v>5175.4</v>
       </c>
       <c r="H277" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="278">
@@ -8303,13 +8291,13 @@
         <v>287</v>
       </c>
       <c r="F281" t="n">
-        <v>21679</v>
+        <v>21676</v>
       </c>
       <c r="G281" t="n">
-        <v>15292.36</v>
+        <v>17579.65</v>
       </c>
       <c r="H281" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="282">
@@ -8325,13 +8313,13 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>3235.89</v>
+        <v>3230.47</v>
       </c>
       <c r="E282" t="n">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="F282" t="n">
-        <v>45682</v>
+        <v>45679</v>
       </c>
       <c r="G282" t="n">
         <v>18725.43</v>
@@ -8359,7 +8347,7 @@
         <v>386</v>
       </c>
       <c r="F283" t="n">
-        <v>41402</v>
+        <v>41399</v>
       </c>
       <c r="G283" t="n">
         <v>24630.68</v>
@@ -8387,7 +8375,7 @@
         <v>116</v>
       </c>
       <c r="F284" t="n">
-        <v>22102</v>
+        <v>22101</v>
       </c>
       <c r="G284" t="n">
         <v>2200</v>
@@ -8443,13 +8431,13 @@
         <v>375</v>
       </c>
       <c r="F286" t="n">
-        <v>75584</v>
+        <v>75582</v>
       </c>
       <c r="G286" t="n">
         <v>12874.56</v>
       </c>
       <c r="H286" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="287">
@@ -8474,10 +8462,10 @@
         <v>6210</v>
       </c>
       <c r="G287" t="n">
-        <v>2287.29</v>
+        <v>4574.58</v>
       </c>
       <c r="H287" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="288">
@@ -8499,7 +8487,7 @@
         <v>444</v>
       </c>
       <c r="F288" t="n">
-        <v>95999</v>
+        <v>95997</v>
       </c>
       <c r="G288" t="n">
         <v>23328.79</v>
@@ -8558,10 +8546,10 @@
         <v>26300</v>
       </c>
       <c r="G290" t="n">
-        <v>13892.37</v>
+        <v>15501.69</v>
       </c>
       <c r="H290" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="291">
@@ -8586,10 +8574,10 @@
         <v>3629</v>
       </c>
       <c r="G291" t="n">
-        <v>2592.37</v>
+        <v>12758.49</v>
       </c>
       <c r="H291" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="292">
@@ -8807,7 +8795,7 @@
         <v>368</v>
       </c>
       <c r="F299" t="n">
-        <v>42894</v>
+        <v>42892</v>
       </c>
       <c r="G299" t="n">
         <v>11858.48</v>
@@ -8831,42 +8819,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -9062,10 +9050,10 @@
         <v>90745</v>
       </c>
       <c r="G8" t="n">
-        <v>21044.08</v>
+        <v>18629.67</v>
       </c>
       <c r="H8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -9781,10 +9769,10 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1496.18</v>
+        <v>1494.66</v>
       </c>
       <c r="E34" t="n">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F34" t="n">
         <v>96893</v>
@@ -10199,51 +10187,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
@@ -10427,7 +10415,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>115706</v>
+        <v>115705</v>
       </c>
       <c r="E7" t="n">
         <v>427</v>
@@ -10757,16 +10745,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4583</v>
+        <v>4381</v>
       </c>
       <c r="E17" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F17" t="n">
-        <v>188.4726260395895</v>
+        <v>180.160861482539</v>
       </c>
       <c r="G17" t="n">
-        <v>3891.744355546909</v>
+        <v>3869.572122693819</v>
       </c>
       <c r="H17" t="n">
         <v>1</v>
@@ -10786,23 +10774,23 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>B0CKHVHVQ1</t>
+          <t>B0BPLWW72Y</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>37123</v>
+        <v>1839</v>
       </c>
       <c r="E18" t="n">
-        <v>172</v>
+        <v>9</v>
       </c>
       <c r="F18" t="n">
-        <v>1526.727373960411</v>
+        <v>75.64142797723062</v>
       </c>
       <c r="G18" t="n">
-        <v>31525.17564445309</v>
+        <v>1624.658977609364</v>
       </c>
       <c r="H18" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -10814,28 +10802,28 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AudioArray - Podcast Mic  SB - KT</t>
+          <t>AudioArray - Conference Mic - SB - AD</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B0CKHVHVQ1</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>13143</v>
+        <v>35486</v>
       </c>
       <c r="E19" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F19" t="n">
-        <v>1517.123893703628</v>
+        <v>1459.39771054023</v>
       </c>
       <c r="G19" t="n">
-        <v>10678.74235735164</v>
+        <v>31345.56889969682</v>
       </c>
       <c r="H19" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -10852,23 +10840,23 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>B0CH4RNWJX</t>
+          <t>B0B4DPX2J2</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3042</v>
+        <v>13143</v>
       </c>
       <c r="E20" t="n">
-        <v>38</v>
+        <v>163</v>
       </c>
       <c r="F20" t="n">
-        <v>351.1759529930117</v>
+        <v>1517.123893703628</v>
       </c>
       <c r="G20" t="n">
-        <v>2471.859773399887</v>
+        <v>10678.74235735164</v>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -10885,20 +10873,20 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>B0FJS57732</t>
+          <t>B0CH4RNWJX</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>3468</v>
+        <v>3042</v>
       </c>
       <c r="E21" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F21" t="n">
-        <v>400.3601533033607</v>
+        <v>351.1759529930117</v>
       </c>
       <c r="G21" t="n">
-        <v>2818.057869248474</v>
+        <v>2471.859773399887</v>
       </c>
       <c r="H21" t="n">
         <v>1</v>
@@ -10913,25 +10901,25 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>AudioArray - Voice Amplifier - SB - KT</t>
+          <t>AudioArray - Podcast Mic  SB - KT</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>B0G39ZHDYP</t>
+          <t>B0FJS57732</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3985</v>
+        <v>3468</v>
       </c>
       <c r="E22" t="n">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="F22" t="n">
-        <v>149.4322574703524</v>
+        <v>400.3601533033607</v>
       </c>
       <c r="G22" t="n">
-        <v>1016.1</v>
+        <v>2818.057869248474</v>
       </c>
       <c r="H22" t="n">
         <v>1</v>
@@ -10951,23 +10939,23 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>B0G3B152FR</t>
+          <t>B0G39ZHDYP</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>12625</v>
+        <v>3985</v>
       </c>
       <c r="E23" t="n">
-        <v>76</v>
+        <v>24</v>
       </c>
       <c r="F23" t="n">
-        <v>473.3477425296476</v>
+        <v>149.4322574703524</v>
       </c>
       <c r="G23" t="n">
-        <v>3218.64</v>
+        <v>1402.246505334448</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -10979,28 +10967,28 @@
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AudioArray_Audio Mixers_SB_Collection</t>
+          <t>AudioArray - Voice Amplifier - SB - KT</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>B0G53H49BS</t>
+          <t>B0G3B152FR</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3512</v>
+        <v>12625</v>
       </c>
       <c r="E24" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F24" t="n">
-        <v>404.375883480471</v>
+        <v>473.3477425296476</v>
       </c>
       <c r="G24" t="n">
-        <v>2372.030000000001</v>
+        <v>4441.813494665551</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -11017,23 +11005,23 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>B0G53M9258</t>
+          <t>B0G53H49BS</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>7527</v>
+        <v>3512</v>
       </c>
       <c r="E25" t="n">
-        <v>172</v>
+        <v>80</v>
       </c>
       <c r="F25" t="n">
-        <v>866.6865739583253</v>
+        <v>404.375883480471</v>
       </c>
       <c r="G25" t="n">
-        <v>5083.900000000001</v>
+        <v>2372.03</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -11050,23 +11038,23 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>B0GXPBHDRF</t>
+          <t>B0G53M9258</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>17563</v>
+        <v>7527</v>
       </c>
       <c r="E26" t="n">
-        <v>400</v>
+        <v>172</v>
       </c>
       <c r="F26" t="n">
-        <v>2022.317542561204</v>
+        <v>866.6865739583252</v>
       </c>
       <c r="G26" t="n">
-        <v>11862.72</v>
+        <v>5083.9</v>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -11078,28 +11066,28 @@
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AudioArray_B0BPLZ5CGV_Audio Interface AI04_SB_ KT</t>
+          <t>AudioArray_Audio Mixers_SB_Collection</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>B0B4G19R58</t>
+          <t>B0GXPBHDRF</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>9935</v>
+        <v>17563</v>
       </c>
       <c r="E27" t="n">
-        <v>69</v>
+        <v>400</v>
       </c>
       <c r="F27" t="n">
-        <v>433.8935309973045</v>
+        <v>2022.317542561204</v>
       </c>
       <c r="G27" t="n">
-        <v>5016.458733085017</v>
+        <v>11862.72</v>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -11116,23 +11104,23 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>B0BPLZ5CGV</t>
+          <t>B0B4G19R58</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>12551</v>
+        <v>9935</v>
       </c>
       <c r="E28" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="F28" t="n">
-        <v>548.1064690026955</v>
+        <v>433.8935309973045</v>
       </c>
       <c r="G28" t="n">
-        <v>6336.931266914982</v>
+        <v>5016.458733085017</v>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -11144,28 +11132,28 @@
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>AudioArray_B0G3Q59X8C_Wireless Mic_SB_KT</t>
+          <t>AudioArray_B0BPLZ5CGV_Audio Interface AI04_SB_ KT</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>B0G3Q59X8C</t>
+          <t>B0BPLZ5CGV</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>9868</v>
+        <v>12551</v>
       </c>
       <c r="E29" t="n">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="F29" t="n">
-        <v>453.13</v>
+        <v>548.1064690026955</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>6336.931266914982</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -11177,28 +11165,28 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>AudioArray_B0GKPXQ8G3_Wireless Mic_SB_KT</t>
+          <t>AudioArray_B0G3Q59X8C_Wireless Mic_SB_KT</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>B0GKPXQ8G3</t>
+          <t>B0G3Q59X8C</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>35101</v>
+        <v>9868</v>
       </c>
       <c r="E30" t="n">
-        <v>208</v>
+        <v>60</v>
       </c>
       <c r="F30" t="n">
-        <v>1501.41</v>
+        <v>453.13</v>
       </c>
       <c r="G30" t="n">
-        <v>2880.51</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -11210,30 +11198,63 @@
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
+          <t>AudioArray_B0GKPXQ8G3_Wireless Mic_SB_KT</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>B0GKPXQ8G3</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>35101</v>
+      </c>
+      <c r="E31" t="n">
+        <v>208</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1501.41</v>
+      </c>
+      <c r="G31" t="n">
+        <v>2880.51</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>AudioArray_B0GN97RFPR_Studio Monitor_SB_KT</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>B0GN97RFPR</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D32" t="n">
         <v>41407</v>
       </c>
-      <c r="E31" t="n">
+      <c r="E32" t="n">
         <v>333</v>
       </c>
-      <c r="F31" t="n">
+      <c r="F32" t="n">
         <v>1669.5</v>
       </c>
-      <c r="G31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" t="inlineStr">
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
         <is>
           <t>Audio Array</t>
         </is>

</xml_diff>